<commit_message>
employee import: per-employee PIN reporting, leading-zero PIN rule; punch demo fixture
</commit_message>
<xml_diff>
--- a/fixtures/employees_sample.xlsx
+++ b/fixtures/employees_sample.xlsx
@@ -551,7 +551,6 @@
           <t>0090</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Lim Wei Sheng</t>
@@ -577,7 +576,6 @@
           <t>12/03/2018</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>90</t>
@@ -593,7 +591,6 @@
           <t>0142</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Nurul Aisyah binti Rahman</t>
@@ -619,10 +616,9 @@
           <t>05/07/2019</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0142</t>
+          <t>142</t>
         </is>
       </c>
     </row>
@@ -635,7 +631,6 @@
           <t>0657</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Tan Chee Keong</t>
@@ -661,7 +656,6 @@
           <t>21/11/2015</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>657</t>
@@ -727,7 +721,6 @@
           <t>1042</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Siti Zubaidah binti Osman</t>
@@ -753,8 +746,6 @@
           <t>17/09/2021</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -765,7 +756,6 @@
           <t>1288</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Wong Mei Ling</t>
@@ -791,7 +781,6 @@
           <t>04/04/2016</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>1288</t>
@@ -807,7 +796,6 @@
           <t>1627</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Aung Ko Min</t>
@@ -833,7 +821,6 @@
           <t>13/02/2023</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>1627</t>
@@ -879,12 +866,8 @@
           <t>08/08/2024</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="D15" t="inlineStr">
         <is>

</xml_diff>